<commit_message>
Thème 2 — LOT 07 : Programmer le lampadaire (îlot 5e_C6 complet) — C4 et C6 de 5e bouclés
Séquence 3 séances sur l'objet-fil du LOT 05 : carte d'identité du programme
par blocs (C6.1), traduction en algorithme en langage naturel (C6.2),
simulateur PARAMÉTRABLE avec mission mairie et verrou expérientiel (C6.3).
QCM 30 q (10/10/10, 2 illustrées, réponses 7/7/8/8, en-tête standard),
synthèses ×2, fiche, matrice, 2 SVG CC0, READMEs C6.2/C6.3.
nouveautes +3 · OVERLAY · index · classeur de progression 5e câblé (S4) ·
tests Playwright 23/23.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016dGiYbQuJoKviTTMpB4BED
</commit_message>
<xml_diff>
--- a/_progressions/5e/Progression_Techno_5e_2026-2027_Martinique.xlsx
+++ b/_progressions/5e/Progression_Techno_5e_2026-2027_Martinique.xlsx
@@ -69,7 +69,7 @@
     <t xml:space="preserve">38</t>
   </si>
   <si>
-    <t xml:space="preserve">2 (+1 partielle)</t>
+    <t xml:space="preserve">4 (5e complet C4+C6)</t>
   </si>
   <si>
     <t xml:space="preserve">Séquences</t>
@@ -1626,7 +1626,7 @@
     <t xml:space="preserve">Séance 1 🔁 (simulateur maison) · 2 🏫 (données/descripteurs) · 3-4 🏫 (programme par blocs) · 5 🏠 QCM + 🏫 éval.</t>
   </si>
   <si>
-    <t xml:space="preserve">✅ Séquence + QCM 32 q + synthèses (C4.5-C4.6) · 🔜 Îlot 5e_C6 (Fable, même objet-fil)</t>
+    <t xml:space="preserve">✅ Séquence + QCM 32 q (C4.5-C4.6) · ✅ « Programmer le lampadaire » (C6.1-C6.3, LOT 07 : séquence + QCM 30 q + synthèses)</t>
   </si>
   <si>
     <t xml:space="preserve">Prob. 4 p.31-36 (système automatisé) · Prob. 7 p.51-58 (programmer une fonctionnalité) · PM 7 p.92</t>
@@ -1933,7 +1933,7 @@
     <t xml:space="preserve">GÉNÉRATEUR DE SÉQUENCE 2024 — S4 · Le lampadaire intelligent (1) : chaîne d'information, données et premiers programmes</t>
   </si>
   <si>
-    <t xml:space="preserve">Thème 2 · P2/P3 · 5 séances de 1 h 30 · Responsable : Fable (Th. 2) · Séances 1-2 : ressources ✅ en ligne · séances 3-5 : îlot 5e_C6 🔜 (même objet-fil)</t>
+    <t xml:space="preserve">Thème 2 · P2/P3 · 5 séances de 1 h 30 · Responsable : Fable (Th. 2) · ✅ TOUTES les ressources en ligne (îlots 5e_C4 + 5e_C6) — séquence 100 % outillée</t>
   </si>
   <si>
     <t xml:space="preserve">La mairie a installé des lampadaires solaires sur le parking du collège ; l'un reste allumé en plein jour, un autre ne s'allume plus. Le club techno doit expliquer comment ils « décident » et aider la mairie à les suivre à distance.</t>
@@ -1975,16 +1975,16 @@
     <t xml:space="preserve">Séances 3-4</t>
   </si>
   <si>
-    <t xml:space="preserve">🔜 avec l'îlot 5e_C6 (même objet-fil)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">🔜 avec l'îlot 5e_C6</t>
+    <t xml:space="preserve">✅ « Programmer le lampadaire » (LOT 07)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">✅ LOT 07</t>
   </si>
   <si>
     <t xml:space="preserve">Séances 4-5</t>
   </si>
   <si>
-    <t xml:space="preserve">🔜 avec l'îlot 5e_C6 + évaluation sommative</t>
+    <t xml:space="preserve">✅ LOT 07 + évaluation sommative</t>
   </si>
   <si>
     <t xml:space="preserve">■ Séance 1 — semaine S13 — 🔁 Hybride — La chaîne d'information du lampadaire</t>
@@ -2035,7 +2035,7 @@
     <t xml:space="preserve">Quelles données le programme du lampadaire utilise-t-il et produit-il ?</t>
   </si>
   <si>
-    <t xml:space="preserve">Îlot 5e_C6 (🔜 en production — même objet-fil) : identifier les données du programme par blocs du lampadaire. En attendant : Nathan Prob. 4 p.31-36 (système automatisé) + Prob. 7 p.52-54.</t>
+    <t xml:space="preserve">Séquence en ligne « Programmer le lampadaire », activité 1 : carte d'identité du programme par blocs (données utilisées/produites/paramètres). https://pll-process.github.io/en-ligne-pour-le-cycle-4/theme-2-structure-fonctionnement-comportement/C6-comprendre-et-modifier-un-programme-associe/5e/5e_C6.1/sequence_5e_C6.1-C6.3_programmer_lampadaire.html</t>
   </si>
   <si>
     <t xml:space="preserve">Investigation guidée ; programme par blocs vidéoprojeté.</t>
@@ -2047,7 +2047,7 @@
     <t xml:space="preserve">Séance 3 : le programme du lampadaire — quelles données entrent (capteurs), quelles données sortent (ordres à la LED). Activités du cahier Nathan p.31-36 / p.52-54.</t>
   </si>
   <si>
-    <t xml:space="preserve">Relire la trace écrite ; terminer l'activité du cahier Nathan commencée en classe (p.54). [Lien de la séquence en ligne 5e_C6 : sera ajouté dès sa mise en ligne.]</t>
+    <t xml:space="preserve">Terminer l'activité 1 (carte d'identité du programme) en ligne : https://pll-process.github.io/en-ligne-pour-le-cycle-4/theme-2-structure-fonctionnement-comportement/C6-comprendre-et-modifier-un-programme-associe/5e/5e_C6.1/sequence_5e_C6.1-C6.3_programmer_lampadaire.html ≈ 20 min, faisable sur téléphone.</t>
   </si>
   <si>
     <t xml:space="preserve">■ Séance 4 — semaine S17 — 🏫 En classe — Modifier une fonctionnalité (5e_C6.2, C6.3)</t>
@@ -2056,7 +2056,7 @@
     <t xml:space="preserve">Comment changer le comportement du lampadaire sans le démonter ?</t>
   </si>
   <si>
-    <t xml:space="preserve">Îlot 5e_C6 (🔜) : modifier un paramètre du programme par blocs (durée de la pleine puissance, seuil nuit) et tester. Nathan Prob. 7 p.55-58 (programmer l'inclinaison d'un vélo).</t>
+    <t xml:space="preserve">Séquence en ligne, activités 2-3 : traduire en algorithme en langage naturel, puis simulateur paramétrable (mission mairie : seuil &gt; 45, verrou expérientiel). https://pll-process.github.io/en-ligne-pour-le-cycle-4/theme-2-structure-fonctionnement-comportement/C6-comprendre-et-modifier-un-programme-associe/5e/5e_C6.1/sequence_5e_C6.1-C6.3_programmer_lampadaire.html · Nathan Prob. 7 p.55-58 en complément.</t>
   </si>
   <si>
     <t xml:space="preserve">Résolution de problème en binômes sur postes (VittaScience / Scratch).</t>
@@ -2068,7 +2068,7 @@
     <t xml:space="preserve">Séance 4 : modifier une fonctionnalité du programme (seuil, durée) et tester. Démarche : je modifie UN paramètre → je teste → je valide. Cahier Nathan p.55-58.</t>
   </si>
   <si>
-    <t xml:space="preserve">Préparer l'évaluation : refaire le QCM complet (32 questions) en mode « Parcours complet » : https://pll-process.github.io/en-ligne-pour-le-cycle-4/theme-2-structure-fonctionnement-comportement/C4-decrire-et-caracteriser-lorganisation/5e/5e_C4.1/qcm_5e_C4.1-C4.8_lampadaire_intelligent.html · relire la synthèse : https://pll-process.github.io/en-ligne-pour-le-cycle-4/theme-2-structure-fonctionnement-comportement/C4-decrire-et-caracteriser-lorganisation/5e/5e_C4.1/Synth%C3%A8ses/synthese_eleve_5e_C4.1-C4.8.html ≈ 30 min, en 2 fois si besoin (la page reprend où tu t'es arrêté).</t>
+    <t xml:space="preserve">Préparer l'évaluation : QCM « Programmer le lampadaire » (30 q) : https://pll-process.github.io/en-ligne-pour-le-cycle-4/theme-2-structure-fonctionnement-comportement/C6-comprendre-et-modifier-un-programme-associe/5e/5e_C6.1/qcm_5e_C6.1-C6.3_programmer_lampadaire.html puis refaire le QCM C4 complet (32 questions) : https://pll-process.github.io/en-ligne-pour-le-cycle-4/theme-2-structure-fonctionnement-comportement/C4-decrire-et-caracteriser-lorganisation/5e/5e_C4.1/qcm_5e_C4.1-C4.8_lampadaire_intelligent.html · relire la synthèse : https://pll-process.github.io/en-ligne-pour-le-cycle-4/theme-2-structure-fonctionnement-comportement/C4-decrire-et-caracteriser-lorganisation/5e/5e_C4.1/Synth%C3%A8ses/synthese_eleve_5e_C4.1-C4.8.html ≈ 30 min, en 2 fois si besoin (la page reprend où tu t'es arrêté).</t>
   </si>
   <si>
     <t xml:space="preserve">■ Séance 5 — semaine S18 — 🏠 puis 🏫 — Bilan et évaluation de la séquence</t>

</xml_diff>

<commit_message>
Thème 2 — LOT 08 : Dépanner le lampadaire (îlot 5e_C5 complet) — la 5e du Thème 2 est bouclée
</commit_message>
<xml_diff>
--- a/_progressions/5e/Progression_Techno_5e_2026-2027_Martinique.xlsx
+++ b/_progressions/5e/Progression_Techno_5e_2026-2027_Martinique.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="🏠 Accueil" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="📅 Calendrier" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="🗓 Frise de l'année" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="📚 Référentiel Cycle 4" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="📗 Référentiel 5e" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="🧭 Progression" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="S1" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="S2" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="S3" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="S4" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="S5" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="S6" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="S7" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="⚙ Moteur" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🏠 Accueil" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📅 Calendrier" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🗓 Frise de l'année" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📚 Référentiel Cycle 4" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📗 Référentiel 5e" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🧭 Progression" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S2" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S3" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S4" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S5" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S6" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S7" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⚙ Moteur" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'📅 Calendrier'!$A$1:$F$52</definedName>
@@ -3898,7 +3898,7 @@
       </c>
       <c r="B14" s="192" t="inlineStr">
         <is>
-          <t>🔜 À produire (Fable — prévu avant le 27/07 si possible, sinon après Conseil)</t>
+          <t>✅ « Dépanner le lampadaire » (C5.1-C5.3, LOT 08 : séquence + QCM 30 q + synthèses + fiche pédagogique)</t>
         </is>
       </c>
       <c r="C14" s="130" t="n"/>
@@ -4059,7 +4059,7 @@
       </c>
       <c r="B25" s="192" t="inlineStr">
         <is>
-          <t>Ateliers tournants : 3 objets en panne « visible » (couture, câble, pièce cassée). Nathan Prob. 5 p.37-40. [Séquence en ligne 🔜 : simulateur de diagnostic 5e.]</t>
+          <t>Ateliers tournants : 3 objets en panne « visible » (couture, câble, pièce cassée). Nathan Prob. 5 p.37-40. [Séquence en ligne ✅ : « Dépanner le lampadaire », inspecteur visuel 6 zones + verrou 6/6.]</t>
         </is>
       </c>
       <c r="C25" s="130" t="n"/>
@@ -4127,7 +4127,7 @@
       </c>
       <c r="B29" s="195" t="inlineStr">
         <is>
-          <t>Cahier Nathan p.38-39 : terminer l'activité d'observation. [Lien séquence en ligne : à ajouter dès mise en ligne.]</t>
+          <t>Cahier Nathan p.38-39 : terminer l'activité d'observation. Séquence en ligne : https://pll-process.github.io/en-ligne-pour-le-cycle-4/theme-2-structure-fonctionnement-comportement/C5-identifier-un-dysfonctionnement-dun-objet/5e/5e_C5.1/sequence_5e_C5.1-C5.3_depanner_lampadaire.html</t>
         </is>
       </c>
       <c r="C29" s="130" t="n"/>
@@ -4313,7 +4313,7 @@
       </c>
       <c r="B43" s="192" t="inlineStr">
         <is>
-          <t>Découverte de l'imprimante 3D du collège (Nathan Point méthode 5 p.90) : du modèle à la pièce. Démonstration d'impression.</t>
+          <t>Découverte de l'imprimante 3D du collège (Nathan Point méthode 5 p.90) : du modèle à la pièce. Démonstration d'impression. [Séance 3 en ligne : l'atelier de la commune, 4 postes, familles additif/enlèvement.]</t>
         </is>
       </c>
       <c r="C43" s="130" t="n"/>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="B47" s="195" t="inlineStr">
         <is>
-          <t>QCM de la séquence en ligne [🔜 lien à ajouter] OU Nathan « Je fais le bilan » p.43. ≈ 15 min.</t>
+          <t>QCM de la séquence en ligne (30 q, corrections détaillées) : https://pll-process.github.io/en-ligne-pour-le-cycle-4/theme-2-structure-fonctionnement-comportement/C5-identifier-un-dysfonctionnement-dun-objet/5e/5e_C5.1/qcm_5e_C5.1-C5.3_depanner_lampadaire.html — OU Nathan « Je fais le bilan » p.43. ≈ 15 min.</t>
         </is>
       </c>
       <c r="C47" s="130" t="n"/>
@@ -7660,8 +7660,8 @@
   <mergeCells count="6">
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="A45:F45"/>
+    <mergeCell ref="A35:F35"/>
     <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A35:F35"/>
     <mergeCell ref="A26:F26"/>
     <mergeCell ref="A20:F20"/>
   </mergeCells>

</xml_diff>